<commit_message>
fix: improve weights extraction and formatting
改進項目：
- 移除 SVORIM_H3 欄位（SVOR 只有兩個 hyperplanes）
- 所有數值四捨五入至小數點後四位
- 修正 Thyroid dataset 的 HCESVM weights 提取（完整 21 個特徵）
- 修正多 dataset 日誌檔案的解析問題
- 新增 dataset 參數支援，正確處理包含多個 datasets 的日誌

技術細節：
- extract_hcesvm_weights() 新增 dataset 參數
- 改進正則表達式以正確匹配多 dataset 日誌
- 所有數值輸出前進行 round(value, 4) 處理

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reports/weights_comparison.xlsx
+++ b/docs/reports/weights_comparison.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,20 +458,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -490,20 +485,19 @@
         <v>-1</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.7818181817489179</v>
+        <v>-0.7818000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.7818181817489179</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-0.7818000000000001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.0978</v>
+      </c>
       <c r="G2" t="n">
-        <v>-0.09777777777477681</v>
+        <v>-0.2769</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.2769230767353361</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.5090909034728398</v>
+        <v>-0.5091</v>
       </c>
     </row>
     <row r="3">
@@ -519,20 +513,19 @@
         <v>-1</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.6363636362493367</v>
+        <v>-0.6364</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.6363636362493367</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>-0.6364</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.08890000000000001</v>
+      </c>
       <c r="G3" t="n">
-        <v>-0.08888888889036246</v>
+        <v>-0.2215</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.2215384612961349</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-0.2909090841428427</v>
+        <v>-0.2909</v>
       </c>
     </row>
     <row r="4">
@@ -548,20 +541,19 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2545454545236617</v>
+        <v>0.2545</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2545454545236617</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0.2545</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0356</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.03555555555491621</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>0.08307692312436574</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1454545421013932</v>
+        <v>0.1455</v>
       </c>
     </row>
     <row r="5">
@@ -577,20 +569,19 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>1.399999999912438</v>
+        <v>1.4</v>
       </c>
       <c r="E5" t="n">
-        <v>1.399999999912438</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>1.4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1956</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.1955555555544913</v>
+        <v>0.4923</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4923076921394549</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.3345454518158136</v>
+        <v>0.3345</v>
       </c>
     </row>
     <row r="6">
@@ -606,20 +597,19 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.672727272748623</v>
+        <v>0.6727</v>
       </c>
       <c r="E6" t="n">
-        <v>0.672727272748623</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0.6727</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.08</v>
+      </c>
       <c r="G6" t="n">
-        <v>0.08000000000034543</v>
+        <v>0.2292</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2292307687412012</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.5236363582963136</v>
+        <v>0.5236</v>
       </c>
     </row>
     <row r="7">
@@ -635,20 +625,19 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>2.218181817937505</v>
+        <v>2.2182</v>
       </c>
       <c r="E7" t="n">
-        <v>2.218181817937505</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>2.2182</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.3467</v>
+      </c>
       <c r="G7" t="n">
-        <v>0.3466666666645393</v>
+        <v>0.78</v>
       </c>
       <c r="H7" t="n">
-        <v>0.779999999782616</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1.381818168333598</v>
+        <v>1.3818</v>
       </c>
     </row>
     <row r="8">
@@ -664,19 +653,18 @@
         <v>-12</v>
       </c>
       <c r="D8" t="n">
-        <v>-9.981818181218793</v>
+        <v>-9.9818</v>
       </c>
       <c r="E8" t="n">
-        <v>-13.6363636354365</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>-13.6364</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.8756</v>
+      </c>
       <c r="G8" t="n">
-        <v>-0.8756</v>
+        <v>-4.0985</v>
       </c>
       <c r="H8" t="n">
-        <v>-4.0985</v>
-      </c>
-      <c r="I8" t="n">
         <v>-6.7891</v>
       </c>
     </row>
@@ -691,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,20 +705,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -749,20 +732,19 @@
         <v>-2</v>
       </c>
       <c r="D2" t="n">
-        <v>-2.000000000019143</v>
+        <v>-2</v>
       </c>
       <c r="E2" t="n">
-        <v>-2.000000000019143</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.24</v>
+      </c>
       <c r="G2" t="n">
-        <v>-0.2399999999998795</v>
+        <v>-1</v>
       </c>
       <c r="H2" t="n">
-        <v>-1.000000000006106</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.2399999999927287</v>
+        <v>-0.24</v>
       </c>
     </row>
     <row r="3">
@@ -778,20 +760,19 @@
         <v>-2</v>
       </c>
       <c r="D3" t="n">
-        <v>-2.000000000019056</v>
+        <v>-2</v>
       </c>
       <c r="E3" t="n">
-        <v>-2.000000000019056</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.24</v>
+      </c>
       <c r="G3" t="n">
-        <v>-0.2400000000004495</v>
+        <v>-1</v>
       </c>
       <c r="H3" t="n">
-        <v>-1.000000000006348</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-0.2399999999941249</v>
+        <v>-0.24</v>
       </c>
     </row>
     <row r="4">
@@ -807,20 +788,19 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>2.000000000019373</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>2.000000000019373</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.24</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.2400000000000391</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1.000000000005499</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.2400000000038792</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="5">
@@ -836,20 +816,19 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2.000000000019148</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>2.000000000019148</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.24</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.2399999999997013</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1.000000000006106</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.239999999982005</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="6">
@@ -865,19 +844,18 @@
         <v>-1</v>
       </c>
       <c r="D6" t="n">
-        <v>1.00000000000056</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>-1.000000000003022</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.76</v>
+      </c>
       <c r="G6" t="n">
-        <v>0.76</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
         <v>-0.76</v>
       </c>
     </row>
@@ -892,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -918,20 +896,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -950,20 +923,19 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.07633587766764333</v>
+        <v>-0.07630000000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.07633587766764333</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-0.07630000000000001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.0276</v>
+      </c>
       <c r="G2" t="n">
-        <v>-0.02758620764754529</v>
+        <v>-0.063</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.06296296281451738</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-3.93347685929799e-12</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="3">
@@ -979,20 +951,19 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2671755665848924</v>
+        <v>0.2672</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2671755665848924</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0.2672</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1743</v>
+      </c>
       <c r="G3" t="n">
-        <v>0.1743213541305278</v>
+        <v>0.2278</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2277777779053416</v>
-      </c>
-      <c r="I3" t="n">
-        <v>2.864799498499428e-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1008,20 +979,19 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01526717201032755</v>
+        <v>0.0153</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01526717201032755</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0.0153</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.008200000000000001</v>
+      </c>
       <c r="G4" t="n">
-        <v>-0.008217173146894772</v>
+        <v>0.0296</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02962962965686744</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3.501923461317121e-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1037,20 +1007,19 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2595419840306374</v>
+        <v>0.2595</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2595419840306374</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>0.2595</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.118</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.1179750578004345</v>
+        <v>0.2204</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2203703698645551</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1.072442144498236e-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1066,20 +1035,19 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.2900763511503425</v>
+        <v>-0.2901</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.2900763511503425</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>-0.2901</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.1197</v>
+      </c>
       <c r="G6" t="n">
-        <v>-0.1197358733636537</v>
+        <v>-0.113</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.112962962988623</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-1.076293722477507e-11</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="7">
@@ -1095,20 +1063,19 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1679389522372528</v>
+        <v>0.1679</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1679389522372528</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>0.1679</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.037</v>
+      </c>
       <c r="G7" t="n">
-        <v>0.03697726541426898</v>
+        <v>0.1796</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1796296291336855</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1.467915915216446e-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1124,20 +1091,19 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1221374006356235</v>
+        <v>0.1221</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1221374006356235</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>0.1221</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0188</v>
+      </c>
       <c r="G8" t="n">
-        <v>0.01878209938448757</v>
+        <v>0.113</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1129629628154616</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1.439198083651506e-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1153,20 +1119,19 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1832061084716946</v>
+        <v>0.1832</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1832061084716946</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>0.1832</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1056</v>
+      </c>
       <c r="G9" t="n">
-        <v>0.1056493006255082</v>
+        <v>0.1889</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1888888889544006</v>
-      </c>
-      <c r="I9" t="n">
-        <v>5.463898407115357e-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1182,20 +1147,19 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.6946564659397474</v>
+        <v>-0.6947</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.6946564659397474</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+        <v>-0.6947</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.2559</v>
+      </c>
       <c r="G10" t="n">
-        <v>-0.2559060925709841</v>
+        <v>-0.3796</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.3796296297050054</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-1.867013025781096e-11</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="11">
@@ -1211,19 +1175,18 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6335878222155574</v>
+        <v>0.6336000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.8015266954979094</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>-0.8015</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.541</v>
+      </c>
       <c r="G11" t="n">
-        <v>0.541</v>
+        <v>-0.4741</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.4741</v>
-      </c>
-      <c r="I11" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1238,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1264,20 +1227,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -1296,20 +1254,19 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-2.510379838599052e-11</v>
+        <v>-0</v>
       </c>
       <c r="E2" t="n">
-        <v>-2.510379838599052e-11</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
       <c r="G2" t="n">
-        <v>1.071169066104153e-11</v>
+        <v>-0</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.703820205310706e-10</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-2.959433533378813e-12</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="3">
@@ -1325,20 +1282,19 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>1.000000000174303</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1.000000000174303</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G3" t="n">
-        <v>0.4000000013061659</v>
+        <v>0.5</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5000000147470565</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.3000000000087354</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4">
@@ -1354,20 +1310,19 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>1.0000000001277</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0000000001277</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.4000000010372765</v>
+        <v>0.5</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5000000139204097</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.3000000000081642</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="5">
@@ -1383,20 +1338,19 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>1.000000000112725</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1.000000000112725</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.4000000009332478</v>
+        <v>0.5</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5000000142838557</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.3000000000032862</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6">
@@ -1412,19 +1366,18 @@
         <v>-9</v>
       </c>
       <c r="D6" t="n">
-        <v>-5.000000000497213</v>
+        <v>-5</v>
       </c>
       <c r="E6" t="n">
-        <v>-7.000000001025012</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>-7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-1.4</v>
+      </c>
       <c r="G6" t="n">
-        <v>-1.4</v>
+        <v>-3</v>
       </c>
       <c r="H6" t="n">
-        <v>-3</v>
-      </c>
-      <c r="I6" t="n">
         <v>-2.8</v>
       </c>
     </row>
@@ -1439,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1465,20 +1418,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -1491,26 +1439,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.0430575714</v>
+        <v>-0.0431</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.122717655</v>
+        <v>-0.1227</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.01594111390691143</v>
+        <v>-0.0159</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.01594111390691143</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-0.0159</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.0114</v>
+      </c>
       <c r="G2" t="n">
-        <v>-0.01140785033058231</v>
+        <v>-0.0117</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.01168467510520189</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.01000745183814508</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="3">
@@ -1520,26 +1467,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-2.9801644896</v>
+        <v>-2.9802</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9052879533</v>
+        <v>0.9053</v>
       </c>
       <c r="D3" t="n">
-        <v>0.08615923077720561</v>
+        <v>0.0862</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08615923077720561</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0.0862</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0617</v>
+      </c>
       <c r="G3" t="n">
-        <v>0.06169382358234165</v>
+        <v>0.0682</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0681658967162494</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-0.1626997287300657</v>
+        <v>-0.1627</v>
       </c>
     </row>
     <row r="4">
@@ -1552,23 +1498,22 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>2.2947273868</v>
+        <v>2.2947</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1020241972923944</v>
+        <v>0.102</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1020241972923944</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0.102</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1634</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.1634451756265729</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>0.06623431794983696</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-0.0120992098966767</v>
+        <v>-0.0121</v>
       </c>
     </row>
     <row r="5">
@@ -1581,23 +1526,22 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>1.6417266103</v>
+        <v>1.6417</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4274334931792914</v>
+        <v>0.4274</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4274334931792914</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>0.4274</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1682</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.1681577700393223</v>
+        <v>0.2912</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2912136276522841</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-0.002092059593721423</v>
+        <v>-0.0021</v>
       </c>
     </row>
     <row r="6">
@@ -1607,26 +1551,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9869375907</v>
+        <v>0.9869</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2680828402</v>
+        <v>0.2681</v>
       </c>
       <c r="D6" t="n">
-        <v>0.060545716164361</v>
+        <v>0.0605</v>
       </c>
       <c r="E6" t="n">
-        <v>0.060545716164361</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0.0605</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0172</v>
+      </c>
       <c r="G6" t="n">
-        <v>0.01719075302779552</v>
+        <v>0.0388</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03878490772428964</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.01698286864706474</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="7">
@@ -1636,25 +1579,24 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14.6990807934</v>
+        <v>14.6991</v>
       </c>
       <c r="C7" t="n">
-        <v>-6.1326207268</v>
+        <v>-6.1326</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.105250740658036</v>
+        <v>-1.1053</v>
       </c>
       <c r="E7" t="n">
-        <v>-2.222684636528864</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>-2.2227</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2342</v>
+      </c>
       <c r="G7" t="n">
-        <v>0.2342</v>
+        <v>-1.0911</v>
       </c>
       <c r="H7" t="n">
-        <v>-1.0911</v>
-      </c>
-      <c r="I7" t="n">
         <v>-1.1011</v>
       </c>
     </row>
@@ -1669,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1695,20 +1637,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -1727,20 +1664,19 @@
         <v>-2</v>
       </c>
       <c r="D2" t="n">
-        <v>-8.264570014790257e-11</v>
+        <v>-0</v>
       </c>
       <c r="E2" t="n">
-        <v>-8.264570014790257e-11</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.5095</v>
+      </c>
       <c r="G2" t="n">
-        <v>-0.5094958014787663</v>
+        <v>-0.7459</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.7459257115574249</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.4000000015041318</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="3">
@@ -1756,20 +1692,19 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>3.326812711375299e-13</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>3.326812711375299e-13</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0033</v>
+      </c>
       <c r="G3" t="n">
-        <v>0.003315590895461627</v>
+        <v>0.0168</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01681543333904547</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3.804133255815483e-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1785,20 +1720,19 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>3.850734569175601e-12</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>3.850734569175601e-12</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0449</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.0449446766272621</v>
+        <v>0.0487</v>
       </c>
       <c r="H4" t="n">
-        <v>0.04871868701387914</v>
-      </c>
-      <c r="I4" t="n">
-        <v>6.990353060570646e-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1814,20 +1748,19 @@
         <v>-2</v>
       </c>
       <c r="D5" t="n">
-        <v>-1.000000000495092</v>
+        <v>-1</v>
       </c>
       <c r="E5" t="n">
-        <v>-1.000000000495092</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.42</v>
+      </c>
       <c r="G5" t="n">
-        <v>-0.4199748471775769</v>
+        <v>-0.7459</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.7459257136818704</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-0.4000000170626499</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="6">
@@ -1843,20 +1776,19 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>2.3841867842877e-14</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2.3841867842877e-14</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.0055</v>
+      </c>
       <c r="G6" t="n">
-        <v>-0.00552598483159269</v>
+        <v>-0.0105</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.01048085229082614</v>
-      </c>
-      <c r="I6" t="n">
-        <v>2.516300492484567e-11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1872,19 +1804,18 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>3.000000001079837</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>1.000000001110825</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.3483</v>
+      </c>
       <c r="G7" t="n">
-        <v>2.3483</v>
+        <v>2.3053</v>
       </c>
       <c r="H7" t="n">
-        <v>2.3053</v>
-      </c>
-      <c r="I7" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -1899,7 +1830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1925,20 +1856,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -1957,20 +1883,19 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0166653341348449</v>
+        <v>0.0167</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0166653341348449</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>0.0167</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0106</v>
+      </c>
       <c r="G2" t="n">
-        <v>0.01062433410327001</v>
+        <v>0.0024</v>
       </c>
       <c r="H2" t="n">
-        <v>0.002425200202025469</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.002425234087608821</v>
+        <v>0.0024</v>
       </c>
     </row>
     <row r="3">
@@ -1986,20 +1911,19 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.006661221785524731</v>
+        <v>0.0067</v>
       </c>
       <c r="E3" t="n">
-        <v>0.006661221785524731</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0.0067</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.007900000000000001</v>
+      </c>
       <c r="G3" t="n">
-        <v>0.007862222917806404</v>
+        <v>0.002</v>
       </c>
       <c r="H3" t="n">
-        <v>0.002042854630981492</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.00204282185779482</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="4">
@@ -2015,20 +1939,19 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0378280702014488</v>
+        <v>0.0378</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0378280702014488</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0.0378</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0225</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.02253349247017474</v>
+        <v>0.0136</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01358460313543153</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.01358446330515936</v>
+        <v>0.0136</v>
       </c>
     </row>
     <row r="5">
@@ -2044,20 +1967,19 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1.801881341701384e-08</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1.801881341701384e-08</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" t="n">
-        <v>1.138224338203248e-10</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>6.305139932377448e-07</v>
-      </c>
-      <c r="I5" t="n">
-        <v>3.748209459008181e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2073,20 +1995,19 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.001881163793325965</v>
+        <v>0.0019</v>
       </c>
       <c r="E6" t="n">
-        <v>0.001881163793325965</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0.0019</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" t="n">
-        <v>3.299060009883089e-10</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.009898111043316655</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.009898227468530413</v>
+        <v>0.009900000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -2102,20 +2023,19 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.00427857170006128</v>
+        <v>-0.0043</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.00427857170006128</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>-0.0043</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.0089</v>
+      </c>
       <c r="G7" t="n">
-        <v>-0.008868649876704162</v>
+        <v>0.0003</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002906113865985701</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.000290500314887924</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="8">
@@ -2131,20 +2051,19 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>3.226707299402416e-08</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>3.226707299402416e-08</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" t="n">
-        <v>2.511538515158352e-10</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>8.43223809412157e-07</v>
-      </c>
-      <c r="I8" t="n">
-        <v>4.567076643910726e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2160,20 +2079,19 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.04308293513906811</v>
+        <v>0.0431</v>
       </c>
       <c r="E9" t="n">
-        <v>0.04308293513906811</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>0.0431</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.014</v>
+      </c>
       <c r="G9" t="n">
-        <v>0.01401034701817083</v>
+        <v>0.0171</v>
       </c>
       <c r="H9" t="n">
-        <v>0.01713153457159202</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.01713153450868806</v>
+        <v>0.0171</v>
       </c>
     </row>
     <row r="10">
@@ -2183,26 +2101,25 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0007429325514651784</v>
+        <v>-0.0007</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0007429325514651784</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+        <v>-0.0007</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" t="n">
-        <v>2.875891702627707e-09</v>
+        <v>-0.0033</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.003336127067975951</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-0.003335972928025863</v>
+        <v>-0.0033</v>
       </c>
     </row>
     <row r="11">
@@ -2211,23 +2128,26 @@
           <t>x10</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
       <c r="D11" t="n">
-        <v>-0.007239047156946284</v>
+        <v>-0.0072</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.007239047156946284</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>-0.0072</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.0183</v>
+      </c>
       <c r="G11" t="n">
-        <v>-0.01830821588001182</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>7.102046698406847e-06</v>
-      </c>
-      <c r="I11" t="n">
-        <v>8.86639478835761e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2236,23 +2156,26 @@
           <t>x11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
       <c r="D12" t="n">
-        <v>-0.0001778007255589107</v>
+        <v>-0.0002</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0001778007255589107</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>-0.0002</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.0113</v>
+      </c>
       <c r="G12" t="n">
-        <v>-0.01130537096905822</v>
+        <v>0.0012</v>
       </c>
       <c r="H12" t="n">
-        <v>0.001237056608583213</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.0012369718543389</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="13">
@@ -2261,23 +2184,26 @@
           <t>x12</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
       <c r="D13" t="n">
-        <v>-5.905072313739691e-05</v>
+        <v>-0.0001</v>
       </c>
       <c r="E13" t="n">
-        <v>-5.905072313739691e-05</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
+        <v>-0.0001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
       <c r="G13" t="n">
-        <v>1.617433061077206e-10</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>1.814783485440066e-07</v>
-      </c>
-      <c r="I13" t="n">
-        <v>6.662087872619783e-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2286,23 +2212,26 @@
           <t>x13</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
       <c r="D14" t="n">
-        <v>1.147627209634759e-08</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>1.147627209634759e-08</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
       <c r="G14" t="n">
-        <v>8.151107274089984e-11</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>2.76372033517256e-07</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1.016920463119457e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2311,23 +2240,26 @@
           <t>x14</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
       <c r="D15" t="n">
-        <v>4.710545115393079e-08</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>4.710545115393079e-08</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" t="n">
-        <v>3.394549942960239e-10</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1.082743382796564e-06</v>
-      </c>
-      <c r="I15" t="n">
-        <v>4.09512194948505e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2336,24 +2268,27 @@
           <t>x15</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
       <c r="D16" t="n">
         <v>-0</v>
       </c>
       <c r="E16" t="n">
         <v>-0</v>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="n">
+        <v>-0</v>
+      </c>
       <c r="G16" t="n">
         <v>-0</v>
       </c>
       <c r="H16" t="n">
         <v>-0</v>
       </c>
-      <c r="I16" t="n">
-        <v>-0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -2361,23 +2296,26 @@
           <t>x16</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
       <c r="D17" t="n">
-        <v>0.0002804283077516376</v>
+        <v>0.0003</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0002804283077516376</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
+        <v>0.0003</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
       <c r="G17" t="n">
-        <v>9.206724497025899e-10</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2.007040280457114e-06</v>
-      </c>
-      <c r="I17" t="n">
-        <v>2.416503420068366e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2386,23 +2324,26 @@
           <t>x17</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
       <c r="D18" t="n">
-        <v>-1.685883946374391</v>
+        <v>-1.6859</v>
       </c>
       <c r="E18" t="n">
-        <v>-1.685883946374391</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
+        <v>-1.6859</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.7383999999999999</v>
+      </c>
       <c r="G18" t="n">
-        <v>-0.7384489735634925</v>
+        <v>-1.0388</v>
       </c>
       <c r="H18" t="n">
-        <v>-1.038762499034644</v>
-      </c>
-      <c r="I18" t="n">
-        <v>-1.038762340810603</v>
+        <v>-1.0388</v>
       </c>
     </row>
     <row r="19">
@@ -2411,23 +2352,26 @@
           <t>x18</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
       <c r="D19" t="n">
-        <v>0.09815848096581557</v>
+        <v>0.0982</v>
       </c>
       <c r="E19" t="n">
-        <v>0.09815848096581557</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
+        <v>0.0982</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.018</v>
+      </c>
       <c r="G19" t="n">
-        <v>0.01795967700641026</v>
+        <v>0.0513</v>
       </c>
       <c r="H19" t="n">
-        <v>0.05126399287065157</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0.05126389307784812</v>
+        <v>0.0513</v>
       </c>
     </row>
     <row r="20">
@@ -2436,23 +2380,26 @@
           <t>x19</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
       <c r="D20" t="n">
-        <v>0.3445822416226599</v>
+        <v>0.3446</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3445822416226599</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
+        <v>0.3446</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.4052</v>
+      </c>
       <c r="G20" t="n">
-        <v>0.4052323829631024</v>
+        <v>0.0598</v>
       </c>
       <c r="H20" t="n">
-        <v>0.05983617494714159</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.05983637697690938</v>
+        <v>0.0598</v>
       </c>
     </row>
     <row r="21">
@@ -2461,23 +2408,26 @@
           <t>x20</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
       <c r="D21" t="n">
-        <v>-0.09614757667356941</v>
+        <v>-0.0961</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.09614757667356941</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
+        <v>-0.0961</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.0689</v>
+      </c>
       <c r="G21" t="n">
-        <v>-0.06889624754343746</v>
+        <v>-0.0206</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.02056487412650785</v>
-      </c>
-      <c r="I21" t="n">
-        <v>-0.02056493986886308</v>
+        <v>-0.0206</v>
       </c>
     </row>
     <row r="22">
@@ -2486,23 +2436,26 @@
           <t>x21</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
       <c r="D22" t="n">
-        <v>0.3916617555718304</v>
+        <v>0.3917</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3916617555718304</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
+        <v>0.3917</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.4634</v>
+      </c>
       <c r="G22" t="n">
-        <v>0.4634325805267661</v>
+        <v>0.0354</v>
       </c>
       <c r="H22" t="n">
-        <v>0.03544873048548611</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.0354490848704426</v>
+        <v>0.0354</v>
       </c>
     </row>
     <row r="23">
@@ -2515,22 +2468,21 @@
         <v>-1</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D23" t="n">
-        <v>0.9539735415934677</v>
+        <v>0.954</v>
       </c>
       <c r="E23" t="n">
-        <v>0.9378111020620062</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
+        <v>0.9378</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.9414</v>
+      </c>
       <c r="G23" t="n">
-        <v>0.9414</v>
+        <v>0.9938</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9938</v>
-      </c>
-      <c r="I23" t="n">
         <v>-0.2062</v>
       </c>
     </row>
@@ -2545,7 +2497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2571,20 +2523,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SVORIM_H3</t>
+          <t>NPSVOR_H1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NPSVOR_H1</t>
+          <t>NPSVOR_H2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>NPSVOR_H2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
@@ -2600,23 +2547,22 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>-1.4486022676</v>
+        <v>-1.4486</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.7232034785724343</v>
+        <v>-0.7232</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.7232034785724343</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>-0.7232</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.2075</v>
+      </c>
       <c r="G2" t="n">
-        <v>-0.2075339851587682</v>
+        <v>-0.1618</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.1618013337259832</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.04392690182461247</v>
+        <v>0.0439</v>
       </c>
     </row>
     <row r="3">
@@ -2626,26 +2572,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2360695535</v>
+        <v>0.2361</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.3857812559</v>
+        <v>-0.3858</v>
       </c>
       <c r="D3" t="n">
-        <v>0.09403756485852138</v>
+        <v>0.094</v>
       </c>
       <c r="E3" t="n">
-        <v>0.09403756485852138</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0.094</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.0716</v>
+      </c>
       <c r="G3" t="n">
-        <v>-0.07156032773096049</v>
+        <v>0.0193</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01926373939023096</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.05546536405576465</v>
+        <v>0.0555</v>
       </c>
     </row>
     <row r="4">
@@ -2658,23 +2603,22 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>-2.3736142565</v>
+        <v>-2.3736</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.7100997253530276</v>
+        <v>-0.7101</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.7100997253530276</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>-0.7101</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.3415</v>
+      </c>
       <c r="G4" t="n">
-        <v>-0.3415433949190761</v>
+        <v>-0.0668</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.06678980472666164</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.3251441223117573</v>
+        <v>0.3251</v>
       </c>
     </row>
     <row r="5">
@@ -2684,26 +2628,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.08377651210000001</v>
+        <v>0.0838</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2745440196</v>
+        <v>0.2745</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2962813919231861</v>
+        <v>0.2963</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2962813919231861</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>0.2963</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0503</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.05025012965310626</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>0.07186684347949809</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.0199880069089657</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="6">
@@ -2713,26 +2656,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0059265751</v>
+        <v>0.0059</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0011989191</v>
+        <v>0.0012</v>
       </c>
       <c r="D6" t="n">
-        <v>0.008241836791475748</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.008241836791475748</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0.008200000000000001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0003</v>
+      </c>
       <c r="G6" t="n">
-        <v>0.000324186222914046</v>
+        <v>0.0034</v>
       </c>
       <c r="H6" t="n">
-        <v>0.003421428658185585</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.002905895988335254</v>
+        <v>0.0029</v>
       </c>
     </row>
     <row r="7">
@@ -2748,20 +2690,19 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2336617833932964</v>
+        <v>0.2337</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2336617833932964</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>0.2337</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2074</v>
+      </c>
       <c r="G7" t="n">
-        <v>0.2074252914472359</v>
+        <v>0.2112</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2111500129184474</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-0.01461091982887882</v>
+        <v>-0.0146</v>
       </c>
     </row>
     <row r="8">
@@ -2771,26 +2712,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-2.6834244583</v>
+        <v>-2.6834</v>
       </c>
       <c r="C8" t="n">
-        <v>-1.1529270227</v>
+        <v>-1.1529</v>
       </c>
       <c r="D8" t="n">
-        <v>-1.860219576135307</v>
+        <v>-1.8602</v>
       </c>
       <c r="E8" t="n">
-        <v>-1.860219576135307</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>-1.8602</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-0.2256</v>
+      </c>
       <c r="G8" t="n">
-        <v>-0.22563844720691</v>
+        <v>-0.5527</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.5526990643547416</v>
-      </c>
-      <c r="I8" t="n">
-        <v>-0.669856406131666</v>
+        <v>-0.6699000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -2806,20 +2746,19 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1853520539241602</v>
+        <v>-0.1854</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1853520539241602</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>-0.1854</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2349</v>
+      </c>
       <c r="G9" t="n">
-        <v>0.2349240786421172</v>
+        <v>-0.4355</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.435488440728942</v>
-      </c>
-      <c r="I9" t="n">
-        <v>-0.3056826067874552</v>
+        <v>-0.3057</v>
       </c>
     </row>
     <row r="10">
@@ -2835,20 +2774,19 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2230201113858764</v>
+        <v>0.223</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2230201113858764</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+        <v>0.223</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1206</v>
+      </c>
       <c r="G10" t="n">
-        <v>0.1206320308057436</v>
+        <v>0.1179</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1178860159088692</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-0.08916810293097067</v>
+        <v>-0.0892</v>
       </c>
     </row>
     <row r="11">
@@ -2858,26 +2796,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.5172678429999999</v>
+        <v>0.5173</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0911356923</v>
+        <v>0.0911</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5109852934063434</v>
+        <v>0.511</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5109852934063434</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>0.511</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.026</v>
+      </c>
       <c r="G11" t="n">
-        <v>0.02601870458662216</v>
+        <v>0.157</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1569568483238347</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.05859656097035022</v>
+        <v>0.0586</v>
       </c>
     </row>
     <row r="12">
@@ -2893,20 +2830,19 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.6377079083383023</v>
+        <v>-0.6377</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.6377079083383023</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>-0.6377</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.1433</v>
+      </c>
       <c r="G12" t="n">
-        <v>-0.1432528056849016</v>
+        <v>-0.1853</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1852619772491062</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-0.2537917991171658</v>
+        <v>-0.2538</v>
       </c>
     </row>
     <row r="13">
@@ -2919,23 +2855,22 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.4213970462</v>
+        <v>-0.4214</v>
       </c>
       <c r="D13" t="n">
-        <v>-1.11594453282502</v>
+        <v>-1.1159</v>
       </c>
       <c r="E13" t="n">
-        <v>-1.11594453282502</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
+        <v>-1.1159</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-0.2191</v>
+      </c>
       <c r="G13" t="n">
-        <v>-0.2191487821784008</v>
+        <v>-0.3443</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.3443303756887504</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-0.1796409873032334</v>
+        <v>-0.1796</v>
       </c>
     </row>
     <row r="14">
@@ -2945,26 +2880,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-6.73927e-05</v>
+        <v>-0.0001</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.004557179</v>
+        <v>-0.0046</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.00481491514950461</v>
+        <v>-0.0048</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.00481491514950461</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+        <v>-0.0048</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.001</v>
+      </c>
       <c r="G14" t="n">
-        <v>-0.001008809185522763</v>
+        <v>-0.0013</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.001339777749991231</v>
-      </c>
-      <c r="I14" t="n">
-        <v>-2.731427083708531e-05</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="15">
@@ -2974,25 +2908,24 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-2.4814924155</v>
+        <v>-2.4815</v>
       </c>
       <c r="C15" t="n">
-        <v>27.22039034</v>
+        <v>27.2204</v>
       </c>
       <c r="D15" t="n">
-        <v>14.29714536666576</v>
+        <v>14.2971</v>
       </c>
       <c r="E15" t="n">
-        <v>8.721630406541411</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>8.7216</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.5838</v>
+      </c>
       <c r="G15" t="n">
-        <v>4.5838</v>
+        <v>2.2886</v>
       </c>
       <c r="H15" t="n">
-        <v>2.2886</v>
-      </c>
-      <c r="I15" t="n">
         <v>-1.5112</v>
       </c>
     </row>

</xml_diff>

<commit_message>
style: apply professional formatting to weights comparison table
格式更新：
- 移除所有儲存格邊框
- Header (第一列) 保留上下邊框
- 最後一列 (b) 保留下邊框
- 所有文字使用 Times New Roman 字體
- Title 不使用粗體

技術實作：
- 新增 apply_formatting() 函數
- 使用 openpyxl.styles 設定 Font 和 Border
- 在寫入資料後自動套用格式設定

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reports/weights_comparison.xlsx
+++ b/docs/reports/weights_comparison.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,10 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -44,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -58,15 +62,41 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border/>
+    <border>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,235 +466,236 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>-0.7818000000000001</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>-0.7818000000000001</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>-0.0978</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>-0.2769</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>-0.5091</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>-0.6364</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>-0.6364</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>-0.08890000000000001</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>-0.2215</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>-0.2909</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>0.2545</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.2545</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.0356</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.08309999999999999</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.1455</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>1.4</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>1.4</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.1956</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.4923</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.3345</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>x5</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="5" t="n">
         <v>0.6727</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="5" t="n">
         <v>0.6727</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.2292</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="5" t="n">
         <v>0.5236</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>x6</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="5" t="n">
         <v>2.2182</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="n">
         <v>2.2182</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.3467</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="5" t="n">
         <v>1.3818</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="7" t="n">
         <v>-17</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="7" t="n">
         <v>-12</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="7" t="n">
         <v>-9.9818</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="7" t="n">
         <v>-13.6364</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="7" t="n">
         <v>-0.8756</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="7" t="n">
         <v>-4.0985</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="7" t="n">
         <v>-6.7891</v>
       </c>
     </row>
@@ -683,179 +714,180 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>-0.24</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>-0.24</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>-0.24</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>-0.24</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.24</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.24</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.24</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="7" t="n">
         <v>-1</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="7" t="n">
         <v>-1</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="7" t="n">
         <v>0.76</v>
       </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
+      <c r="G6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="n">
         <v>-0.76</v>
       </c>
     </row>
@@ -874,319 +906,320 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5" t="n">
         <v>-0.07630000000000001</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>-0.07630000000000001</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>-0.0276</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>-0.063</v>
       </c>
-      <c r="H2" t="n">
-        <v>-0</v>
+      <c r="H2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5" t="n">
         <v>0.2672</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.2672</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.1743</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.2278</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>0.0153</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.0153</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>-0.008200000000000001</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.0296</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="n">
         <v>0.2595</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.2595</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.118</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.2204</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>x5</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>-0.2901</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="5" t="n">
         <v>-0.2901</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="5" t="n">
         <v>-0.1197</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="5" t="n">
         <v>-0.113</v>
       </c>
-      <c r="H6" t="n">
-        <v>-0</v>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>x6</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>0.1679</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="n">
         <v>0.1679</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.037</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.1796</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>x7</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>0.1221</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="5" t="n">
         <v>0.1221</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.0188</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="5" t="n">
         <v>0.113</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>x8</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>0.1832</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="5" t="n">
         <v>0.1832</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.1056</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="5" t="n">
         <v>0.1889</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>x9</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>-0.6947</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="5" t="n">
         <v>-0.6947</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="5" t="n">
         <v>-0.2559</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="5" t="n">
         <v>-0.3796</v>
       </c>
-      <c r="H10" t="n">
-        <v>-0</v>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="7" t="n">
         <v>-1</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="7" t="n">
         <v>0.6336000000000001</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="7" t="n">
         <v>-0.8015</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="7" t="n">
         <v>0.541</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="7" t="n">
         <v>-0.4741</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="7" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1205,179 +1238,180 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>-0</v>
+      <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.4</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.4</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.4</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="7" t="n">
         <v>-7</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="7" t="n">
         <v>-9</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="7" t="n">
         <v>-5</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="7" t="n">
         <v>-7</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="7" t="n">
         <v>-1.4</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="7" t="n">
         <v>-3</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="7" t="n">
         <v>-2.8</v>
       </c>
     </row>
@@ -1396,207 +1430,208 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="5" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="5" t="n">
         <v>-0.1227</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>-0.0159</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>-0.0159</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>-0.0114</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>-0.0117</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>0.01</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>-2.9802</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="5" t="n">
         <v>0.9053</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>0.0862</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.0862</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.0617</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.0682</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>-0.1627</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
         <v>2.2947</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>0.102</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.102</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.1634</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.06619999999999999</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>-0.0121</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="n">
         <v>1.6417</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.4274</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.4274</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.1682</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.2912</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>-0.0021</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>x5</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="5" t="n">
         <v>0.9869</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="5" t="n">
         <v>0.2681</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="5" t="n">
         <v>0.0605</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="5" t="n">
         <v>0.0605</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.0172</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.0388</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="5" t="n">
         <v>0.017</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>14.6991</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="7" t="n">
         <v>-6.1326</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="7" t="n">
         <v>-1.1053</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="7" t="n">
         <v>-2.2227</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="7" t="n">
         <v>0.2342</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="7" t="n">
         <v>-1.0911</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="7" t="n">
         <v>-1.1011</v>
       </c>
     </row>
@@ -1615,207 +1650,208 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="D2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="n">
         <v>-0.5095</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>-0.7459</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>-0.4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="B3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5" t="n">
         <v>0.0033</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.0168</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>0.0449</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.0487</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>-0.42</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>-0.7459</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>-0.4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>x5</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5" t="n">
         <v>-0.0055</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="5" t="n">
         <v>-0.0105</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="7" t="n">
         <v>2.3483</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="7" t="n">
         <v>2.3053</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="7" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -1834,655 +1870,656 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5" t="n">
         <v>0.0167</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>0.0167</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>0.0106</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>0.0024</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>0.0024</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5" t="n">
         <v>0.0067</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.0067</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.007900000000000001</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>0.002</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>0.0378</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.0378</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.0225</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.0136</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.0136</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>x5</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>0.0019</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="5" t="n">
         <v>0.0019</v>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
         <v>0.009900000000000001</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="5" t="n">
         <v>0.009900000000000001</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>x6</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>-0.0043</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="n">
         <v>-0.0043</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="5" t="n">
         <v>-0.0089</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="5" t="n">
         <v>0.0003</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>x7</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>x8</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>0.0431</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="5" t="n">
         <v>0.0431</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.014</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="5" t="n">
         <v>0.0171</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="5" t="n">
         <v>0.0171</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>x9</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>-0.0007</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="5" t="n">
         <v>-0.0007</v>
       </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
         <v>-0.0033</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="5" t="n">
         <v>-0.0033</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>x10</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
         <v>-0.0072</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="5" t="n">
         <v>-0.0072</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="5" t="n">
         <v>-0.0183</v>
       </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>x11</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
         <v>-0.0002</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="5" t="n">
         <v>-0.0002</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="5" t="n">
         <v>-0.0113</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="5" t="n">
         <v>0.0012</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="5" t="n">
         <v>0.0012</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>x12</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
         <v>-0.0001</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="5" t="n">
         <v>-0.0001</v>
       </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>x13</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>x14</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>x15</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>-0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>-0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>-0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>-0</v>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>x16</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>x17</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="n">
         <v>-1.6859</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="5" t="n">
         <v>-1.6859</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="5" t="n">
         <v>-0.7383999999999999</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="5" t="n">
         <v>-1.0388</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H18" s="5" t="n">
         <v>-1.0388</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>x18</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
         <v>0.0982</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="5" t="n">
         <v>0.0982</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="5" t="n">
         <v>0.018</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="5" t="n">
         <v>0.0513</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="5" t="n">
         <v>0.0513</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>x19</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n">
         <v>0.3446</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="5" t="n">
         <v>0.3446</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="5" t="n">
         <v>0.4052</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="5" t="n">
         <v>0.0598</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" s="5" t="n">
         <v>0.0598</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>x20</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
         <v>-0.0961</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="5" t="n">
         <v>-0.0961</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="5" t="n">
         <v>-0.0689</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" s="5" t="n">
         <v>-0.0206</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="5" t="n">
         <v>-0.0206</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>x21</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
         <v>0.3917</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="5" t="n">
         <v>0.3917</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="5" t="n">
         <v>0.4634</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="5" t="n">
         <v>0.0354</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" s="5" t="n">
         <v>0.0354</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="7" t="n">
         <v>-1</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="7" t="n">
         <v>-1</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="7" t="n">
         <v>0.954</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="7" t="n">
         <v>0.9378</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="7" t="n">
         <v>0.9414</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="7" t="n">
         <v>0.9938</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H23" s="7" t="n">
         <v>-0.2062</v>
       </c>
     </row>
@@ -2501,431 +2538,432 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>HCESVM_H2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SVORIM_H2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>NPSVOR_H3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>-1.4486</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>-0.7232</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>-0.7232</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>-0.2075</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>-0.1618</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>0.0439</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>0.2361</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="5" t="n">
         <v>-0.3858</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>0.094</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.094</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>-0.0716</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.0193</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>0.0555</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
         <v>-2.3736</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>-0.7101</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>-0.7101</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>-0.3415</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>-0.0668</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.3251</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="5" t="n">
         <v>0.0838</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="5" t="n">
         <v>0.2745</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.2963</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.2963</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.0503</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.07190000000000001</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>x5</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="5" t="n">
         <v>0.0059</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="5" t="n">
         <v>0.0012</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="5" t="n">
         <v>0.008200000000000001</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="5" t="n">
         <v>0.008200000000000001</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.0034</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="5" t="n">
         <v>0.0029</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>x6</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>0.2337</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="n">
         <v>0.2337</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.2074</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.2112</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="5" t="n">
         <v>-0.0146</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>x7</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="5" t="n">
         <v>-2.6834</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="5" t="n">
         <v>-1.1529</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="5" t="n">
         <v>-1.8602</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="5" t="n">
         <v>-1.8602</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="5" t="n">
         <v>-0.2256</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="5" t="n">
         <v>-0.5527</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="5" t="n">
         <v>-0.6699000000000001</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>x8</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>-0.1854</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="5" t="n">
         <v>-0.1854</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.2349</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="5" t="n">
         <v>-0.4355</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="5" t="n">
         <v>-0.3057</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>x9</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>0.223</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="5" t="n">
         <v>0.223</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="5" t="n">
         <v>0.1206</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="5" t="n">
         <v>0.1179</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="5" t="n">
         <v>-0.0892</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>x10</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="5" t="n">
         <v>0.5173</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="5" t="n">
         <v>0.0911</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="5" t="n">
         <v>0.511</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="5" t="n">
         <v>0.511</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.026</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="5" t="n">
         <v>0.157</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="5" t="n">
         <v>0.0586</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>x11</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
         <v>-0.6377</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="5" t="n">
         <v>-0.6377</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="5" t="n">
         <v>-0.1433</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="5" t="n">
         <v>-0.1853</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="5" t="n">
         <v>-0.2538</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>x12</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="n">
         <v>-0.4214</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="5" t="n">
         <v>-1.1159</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="5" t="n">
         <v>-1.1159</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="5" t="n">
         <v>-0.2191</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="5" t="n">
         <v>-0.3443</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="5" t="n">
         <v>-0.1796</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>x13</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="5" t="n">
         <v>-0.0001</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="5" t="n">
         <v>-0.0046</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="5" t="n">
         <v>-0.0048</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="5" t="n">
         <v>-0.0048</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="5" t="n">
         <v>-0.001</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="5" t="n">
         <v>-0.0013</v>
       </c>
-      <c r="H14" t="n">
-        <v>-0</v>
+      <c r="H14" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="7" t="n">
         <v>-2.4815</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="7" t="n">
         <v>27.2204</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="7" t="n">
         <v>14.2971</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="7" t="n">
         <v>8.7216</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="7" t="n">
         <v>4.5838</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="7" t="n">
         <v>2.2886</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="7" t="n">
         <v>-1.5112</v>
       </c>
     </row>

</xml_diff>